<commit_message>
Add 3 × HEK g1 KO from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/baris.xlsx
+++ b/cellstocks/data/baris.xlsx
@@ -148,6 +148,267 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAro box deneme</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK g1 KO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">myco bilmiyorum</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtr71fv1-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAro box deneme</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK g1 KO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">myco bilmiyorum</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtr71fv1-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAro box deneme</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK g1 KO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">myco bilmiyorum</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtr71fv1-2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -192,6 +453,37 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK g1 KO</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -313,12 +605,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -341,10 +633,10 @@
         <v>81</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Take out HEK g1 KO from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/baris.xlsx
+++ b/cellstocks/data/baris.xlsx
@@ -166,7 +166,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -231,7 +231,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtr71fv1-0</t>
+          <t xml:space="preserve">v-mtr71fv1-1</t>
         </is>
       </c>
     </row>
@@ -253,7 +253,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -318,31 +318,11 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtr71fv1-1</t>
+          <t xml:space="preserve">v-mtr71fv1-2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAro box deneme</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A3</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t xml:space="preserve">HEK g1 KO</t>
@@ -400,12 +380,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtr71fv1-2</t>
+          <t xml:space="preserve">v-mtr71fv1-0</t>
         </is>
       </c>
     </row>
@@ -475,10 +455,10 @@
         </is>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -543,6 +523,53 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK g1 KO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAro box deneme</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtr71fv1-0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -633,10 +660,10 @@
         <v>81</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Confirm 53 dates from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/baris.xlsx
+++ b/cellstocks/data/baris.xlsx
@@ -184,14 +184,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -261,14 +261,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -338,14 +338,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -415,14 +415,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1262,14 +1262,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1339,14 +1339,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-02-10</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t xml:space="preserve">10.02.20</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1570,14 +1570,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-01-01</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.20</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1647,14 +1647,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-01-01</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.20</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1724,14 +1724,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-01-01</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.20</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1801,14 +1801,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-01-01</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.20</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -1878,14 +1878,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-01-01</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">01.01.20</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2678,14 +2678,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-09-04</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t xml:space="preserve">04.09.20</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2755,14 +2755,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-09-04</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t xml:space="preserve">04.09.20</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2832,14 +2832,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-09-04</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t xml:space="preserve">04.09.20</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2909,14 +2909,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-06</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t xml:space="preserve">06.08.20</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2986,14 +2986,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-06</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">06.08.20</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3063,14 +3063,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3145,14 +3145,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3227,14 +3227,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3309,14 +3309,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3391,14 +3391,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3473,14 +3473,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-08-01</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t xml:space="preserve">01.08.20</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -4094,14 +4094,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-08</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t xml:space="preserve">08.07.20</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4171,14 +4171,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-08</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t xml:space="preserve">08.07.20</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4248,14 +4248,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-08</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t xml:space="preserve">08.07.20</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4325,14 +4325,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-08</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t xml:space="preserve">08.07.20</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -5125,14 +5125,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-10</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.20</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -5202,14 +5202,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-10</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.20</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -5279,14 +5279,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-10</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.20</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -5818,14 +5818,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-10</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.20</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5895,14 +5895,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-07-10</t>
+        </is>
+      </c>
       <c r="I75" t="inlineStr">
         <is>
           <t xml:space="preserve">10.07.20</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -5972,14 +5972,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -6054,14 +6054,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -6136,14 +6136,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I78" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6218,14 +6218,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I79" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -6300,14 +6300,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I80" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -6382,14 +6382,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2020-03-02</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t xml:space="preserve">02.03.20</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -7100,14 +7100,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-11</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t xml:space="preserve">11.06.21</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -7592,14 +7592,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-07</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t xml:space="preserve">07.06.21</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -7674,14 +7674,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-07</t>
+        </is>
+      </c>
       <c r="I97" t="inlineStr">
         <is>
           <t xml:space="preserve">07.06.21</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -7756,14 +7756,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-07</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr">
         <is>
           <t xml:space="preserve">07.06.21</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -7838,14 +7838,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-07</t>
+        </is>
+      </c>
       <c r="I99" t="inlineStr">
         <is>
           <t xml:space="preserve">07.06.21</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -7920,14 +7920,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021-06-07</t>
+        </is>
+      </c>
       <c r="I100" t="inlineStr">
         <is>
           <t xml:space="preserve">07.06.21</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -37727,14 +37727,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-12</t>
+        </is>
+      </c>
       <c r="I506" t="inlineStr">
         <is>
           <t xml:space="preserve">12.10.23</t>
-        </is>
-      </c>
-      <c r="J506" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K506" t="inlineStr">
@@ -37809,14 +37809,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-12</t>
+        </is>
+      </c>
       <c r="I507" t="inlineStr">
         <is>
           <t xml:space="preserve">12.10.23</t>
-        </is>
-      </c>
-      <c r="J507" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K507" t="inlineStr">
@@ -37891,14 +37891,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-10-12</t>
+        </is>
+      </c>
       <c r="I508" t="inlineStr">
         <is>
           <t xml:space="preserve">12.10.23</t>
-        </is>
-      </c>
-      <c r="J508" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K508" t="inlineStr">
@@ -38055,14 +38055,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I510" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J510" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K510" t="inlineStr">
@@ -38137,14 +38137,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I511" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J511" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K511" t="inlineStr">
@@ -38219,14 +38219,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I512" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J512" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K512" t="inlineStr">
@@ -38301,14 +38301,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I513" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J513" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K513" t="inlineStr">
@@ -38383,14 +38383,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I514" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J514" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K514" t="inlineStr">
@@ -38465,14 +38465,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I515" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J515" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K515" t="inlineStr">
@@ -38547,14 +38547,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-11-02</t>
+        </is>
+      </c>
       <c r="I516" t="inlineStr">
         <is>
           <t xml:space="preserve">02.11.23</t>
-        </is>
-      </c>
-      <c r="J516" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K516" t="inlineStr">

</xml_diff>

<commit_message>
Add a resistance rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/baris.xlsx
+++ b/cellstocks/data/baris.xlsx
@@ -3210,7 +3210,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -8584,7 +8584,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -9046,7 +9046,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -11192,7 +11192,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -11269,7 +11269,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -12779,7 +12779,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -13241,7 +13241,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -13472,7 +13472,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -14823,7 +14823,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -15054,7 +15054,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -15131,7 +15131,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -18397,7 +18397,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -20533,7 +20533,7 @@
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
@@ -20893,7 +20893,7 @@
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N268" t="inlineStr">
@@ -21253,7 +21253,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N273" t="inlineStr">
@@ -21469,7 +21469,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -21613,7 +21613,7 @@
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N278" t="inlineStr">
@@ -22189,7 +22189,7 @@
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N286" t="inlineStr">
@@ -22688,7 +22688,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -22976,7 +22976,7 @@
       </c>
       <c r="M297" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
@@ -23264,7 +23264,7 @@
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N301" t="inlineStr">
@@ -23974,7 +23974,7 @@
       </c>
       <c r="M311" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N311" t="inlineStr">
@@ -24617,7 +24617,7 @@
       </c>
       <c r="M320" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N320" t="inlineStr">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="M341" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N341" t="inlineStr">
@@ -28162,7 +28162,7 @@
       </c>
       <c r="M370" t="inlineStr">
         <is>
-          <t xml:space="preserve">CisR</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N370" t="inlineStr">
@@ -29093,7 +29093,7 @@
       </c>
       <c r="M383" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N383" t="inlineStr">
@@ -29381,7 +29381,7 @@
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N387" t="inlineStr">
@@ -29453,7 +29453,7 @@
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
@@ -29597,7 +29597,7 @@
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
@@ -29741,7 +29741,7 @@
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
@@ -30029,7 +30029,7 @@
       </c>
       <c r="M396" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N396" t="inlineStr">
@@ -30173,7 +30173,7 @@
       </c>
       <c r="M398" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N398" t="inlineStr">
@@ -30317,7 +30317,7 @@
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
@@ -30677,7 +30677,7 @@
       </c>
       <c r="M405" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N405" t="inlineStr">
@@ -30749,7 +30749,7 @@
       </c>
       <c r="M406" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N406" t="inlineStr">
@@ -31397,7 +31397,7 @@
       </c>
       <c r="M415" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N415" t="inlineStr">
@@ -31469,7 +31469,7 @@
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N416" t="inlineStr">
@@ -31541,7 +31541,7 @@
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N417" t="inlineStr">
@@ -31896,7 +31896,7 @@
       </c>
       <c r="M422" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N422" t="inlineStr">
@@ -32400,7 +32400,7 @@
       </c>
       <c r="M429" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N429" t="inlineStr">
@@ -32894,7 +32894,7 @@
       </c>
       <c r="M436" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N436" t="inlineStr">
@@ -32966,7 +32966,7 @@
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -33038,7 +33038,7 @@
       </c>
       <c r="M438" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N438" t="inlineStr">
@@ -36052,7 +36052,7 @@
       </c>
       <c r="M480" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N480" t="inlineStr">
@@ -36124,7 +36124,7 @@
       </c>
       <c r="M481" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N481" t="inlineStr">
@@ -36196,7 +36196,7 @@
       </c>
       <c r="M482" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N482" t="inlineStr">
@@ -36268,7 +36268,7 @@
       </c>
       <c r="M483" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N483" t="inlineStr">
@@ -36340,7 +36340,7 @@
       </c>
       <c r="M484" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N484" t="inlineStr">
@@ -36412,7 +36412,7 @@
       </c>
       <c r="M485" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N485" t="inlineStr">
@@ -36484,7 +36484,7 @@
       </c>
       <c r="M486" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N486" t="inlineStr">
@@ -36556,7 +36556,7 @@
       </c>
       <c r="M487" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N487" t="inlineStr">
@@ -36700,7 +36700,7 @@
       </c>
       <c r="M489" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N489" t="inlineStr">
@@ -36772,7 +36772,7 @@
       </c>
       <c r="M490" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N490" t="inlineStr">
@@ -36844,7 +36844,7 @@
       </c>
       <c r="M491" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N491" t="inlineStr">
@@ -36916,7 +36916,7 @@
       </c>
       <c r="M492" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N492" t="inlineStr">
@@ -36988,7 +36988,7 @@
       </c>
       <c r="M493" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N493" t="inlineStr">
@@ -37060,7 +37060,7 @@
       </c>
       <c r="M494" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N494" t="inlineStr">
@@ -37132,7 +37132,7 @@
       </c>
       <c r="M495" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N495" t="inlineStr">
@@ -37204,7 +37204,7 @@
       </c>
       <c r="M496" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N496" t="inlineStr">
@@ -37276,7 +37276,7 @@
       </c>
       <c r="M497" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N497" t="inlineStr">
@@ -37348,7 +37348,7 @@
       </c>
       <c r="M498" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N498" t="inlineStr">
@@ -37420,7 +37420,7 @@
       </c>
       <c r="M499" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N499" t="inlineStr">
@@ -37492,7 +37492,7 @@
       </c>
       <c r="M500" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N500" t="inlineStr">
@@ -37564,7 +37564,7 @@
       </c>
       <c r="M501" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N501" t="inlineStr">
@@ -37636,7 +37636,7 @@
       </c>
       <c r="M502" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">CabaR</t>
         </is>
       </c>
       <c r="N502" t="inlineStr">

</xml_diff>